<commit_message>
fix: update international phone validation, 50 rows limit, and sample file
</commit_message>
<xml_diff>
--- a/public/samples/lead_bulk_upload_sample.xlsx
+++ b/public/samples/lead_bulk_upload_sample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sample Leads" sheetId="1" r:id="rId1"/>
+    <sheet name="Leads" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -64,8 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,54 +398,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:C4"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>full_name</v>
+        <v>Full Name</v>
       </c>
       <c r="B1" t="str">
-        <v>email</v>
+        <v>Email</v>
       </c>
       <c r="C1" t="str">
-        <v>phone</v>
-      </c>
-      <c r="D1" t="str">
-        <v>country</v>
-      </c>
-      <c r="E1" t="str">
-        <v>state</v>
-      </c>
-      <c r="F1" t="str">
-        <v>city</v>
-      </c>
-      <c r="G1" t="str">
-        <v>address_line1</v>
-      </c>
-      <c r="H1" t="str">
-        <v>postal_code</v>
-      </c>
-      <c r="I1" t="str">
-        <v>lead_source</v>
-      </c>
-      <c r="J1" t="str">
-        <v>best_time_to_call</v>
-      </c>
-      <c r="K1" t="str">
-        <v>whatsapp_number</v>
+        <v>Phone</v>
       </c>
     </row>
     <row r="2">
@@ -454,177 +423,35 @@
       <c r="B2" t="str">
         <v>rahul.sharma@example.com</v>
       </c>
-      <c r="C2" t="str">
-        <v>+919876543210</v>
-      </c>
-      <c r="D2" t="str">
-        <v>India</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Maharashtra</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Mumbai</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Flat 402, Sunrise Apt, Andheri West</v>
-      </c>
-      <c r="H2" t="str">
-        <v>400053</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Google Ads</v>
-      </c>
-      <c r="J2" t="str">
-        <v>10:00 AM - 12:00 PM</v>
-      </c>
-      <c r="K2" t="str">
+      <c r="C2" s="1" t="str">
         <v>+919876543210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Priya Patel</v>
+        <v>John Smith</v>
       </c>
       <c r="B3" t="str">
-        <v>priya.patel@example.com</v>
-      </c>
-      <c r="C3" t="str">
-        <v>+919123456780</v>
-      </c>
-      <c r="D3" t="str">
-        <v>India</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Gujarat</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Ahmedabad</v>
-      </c>
-      <c r="G3" t="str">
-        <v>12 Shivalik Heights, SG Highway</v>
-      </c>
-      <c r="H3" t="str">
-        <v>380015</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Facebook</v>
-      </c>
-      <c r="J3" t="str">
-        <v>02:00 PM - 04:00 PM</v>
-      </c>
-      <c r="K3" t="str">
-        <v>+919123456780</v>
+        <v>john.smith@example.com</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>+14155552671</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Amit Verma</v>
+        <v>David Wilson</v>
       </c>
       <c r="B4" t="str">
-        <v>amit.verma@example.com</v>
-      </c>
-      <c r="C4" t="str">
-        <v>+919811223344</v>
-      </c>
-      <c r="D4" t="str">
-        <v>India</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Delhi</v>
-      </c>
-      <c r="F4" t="str">
-        <v>New Delhi</v>
-      </c>
-      <c r="G4" t="str">
-        <v>B-14, Connaught Place</v>
-      </c>
-      <c r="H4" t="str">
-        <v>110001</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Website</v>
-      </c>
-      <c r="J4" t="str">
-        <v>05:00 PM - 07:00 PM</v>
-      </c>
-      <c r="K4" t="str">
-        <v>+919811223344</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Sneha Rao</v>
-      </c>
-      <c r="B5" t="str">
-        <v>sneha.rao@example.com</v>
-      </c>
-      <c r="C5" t="str">
-        <v>+919988776655</v>
-      </c>
-      <c r="D5" t="str">
-        <v>India</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Karnataka</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Bengaluru</v>
-      </c>
-      <c r="G5" t="str">
-        <v>88 Indiranagar 100ft Road</v>
-      </c>
-      <c r="H5" t="str">
-        <v>560038</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Direct Call</v>
-      </c>
-      <c r="J5" t="str">
-        <v>11:00 AM - 01:00 PM</v>
-      </c>
-      <c r="K5" t="str">
-        <v>+919988776655</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>John Doe</v>
-      </c>
-      <c r="B6" t="str">
-        <v>john.doe@example.com</v>
-      </c>
-      <c r="C6" t="str">
-        <v>+12025550143</v>
-      </c>
-      <c r="D6" t="str">
-        <v>USA</v>
-      </c>
-      <c r="E6" t="str">
-        <v>California</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Los Angeles</v>
-      </c>
-      <c r="G6" t="str">
-        <v>742 Evergreen Terrace</v>
-      </c>
-      <c r="H6" t="str">
-        <v>90001</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Referral</v>
-      </c>
-      <c r="J6" t="str">
-        <v>09:00 AM - 11:00 AM</v>
-      </c>
-      <c r="K6" t="str">
-        <v>+12025550143</v>
+        <v>david.wilson@example.com</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>+447911123456</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>